<commit_message>
fix: updated usb script
</commit_message>
<xml_diff>
--- a/Continous_Developement/NFC_Rev3.01_usb_control/NFC_USB_Relay_Implementation_Overview.xlsx
+++ b/Continous_Developement/NFC_Rev3.01_usb_control/NFC_USB_Relay_Implementation_Overview.xlsx
@@ -26,30 +26,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="135">
   <si>
     <t>NFC USB Relay Implementation Overview</t>
   </si>
   <si>
-    <t>Legends</t>
-  </si>
-  <si>
     <t>Purpose: Add external USB relay control for CAPA switch and short operations, separate from firmware variable hacks.</t>
   </si>
   <si>
-    <t>Switches to control by script with logic value 1</t>
-  </si>
-  <si>
     <t>Scope: USB relay helper, automation wrapper, Trace32 adapter integration, GUI manual control, safety controls.</t>
   </si>
   <si>
-    <t>Capacitors controlling by switches through USB</t>
-  </si>
-  <si>
     <t>Status: Implementation completed in code; hardware validation pending with actual relay board.</t>
-  </si>
-  <si>
-    <t>External USB hardware controlled by PC not controleed by Trace32</t>
   </si>
   <si>
     <t>Key Benefits: safer hardware control, independent CAPA relay path, configurable COM parameters, manual test support.</t>
@@ -499,7 +487,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -539,24 +527,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF7030A0"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -656,7 +626,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -668,12 +638,6 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -749,19 +713,19 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>946151</xdr:colOff>
+      <xdr:colOff>19050</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>44450</xdr:rowOff>
+      <xdr:rowOff>31750</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>711200</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>94201</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>387017</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPr id="10" name="Picture 9"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -774,8 +738,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4540251" y="228600"/>
-          <a:ext cx="5003799" cy="3580351"/>
+          <a:off x="3613150" y="215900"/>
+          <a:ext cx="8191167" cy="3771900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1072,69 +1036,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="51.453125" style="3" customWidth="1"/>
     <col min="2" max="4" width="25" style="3" customWidth="1"/>
     <col min="5" max="5" width="16.1796875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="10.54296875" style="3" customWidth="1"/>
-    <col min="7" max="7" width="25" style="3" customWidth="1"/>
-    <col min="8" max="8" width="3.36328125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="3.36328125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F2" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+    </row>
+    <row r="3" spans="1:6" ht="48.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="48.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+    <row r="4" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="6"/>
-      <c r="G3" s="5" t="s">
+    </row>
+    <row r="5" spans="1:6" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+    <row r="6" spans="1:6" ht="99.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
         <v>4</v>
-      </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F5" s="8"/>
-      <c r="G5" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="99.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -1151,97 +1094,97 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="58" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="58" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="58" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1259,104 +1202,104 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1374,86 +1317,86 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1471,100 +1414,100 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>93</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="58" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B7" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D7" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1582,86 +1525,86 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="58" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -1679,129 +1622,129 @@
   <sheetData>
     <row r="1" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="F2" s="16" t="s">
-        <v>126</v>
-      </c>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="K2" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
+      <c r="A2" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="F2" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="K2" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
     </row>
     <row r="3" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="10"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
     </row>
     <row r="4" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="10"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10"/>
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
     </row>
     <row r="5" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="6" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="F6" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="K6" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
+      <c r="A6" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="F6" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="K6" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
     </row>
     <row r="7" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="10"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
     </row>
     <row r="8" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="10"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
     </row>
     <row r="9" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="10" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="11" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
+      <c r="A11" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
     </row>
     <row r="12" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
     </row>
     <row r="13" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
     </row>
     <row r="14" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
     </row>
     <row r="15" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -1832,129 +1775,129 @@
   <sheetData>
     <row r="1" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="20"/>
-      <c r="F2" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="20"/>
-      <c r="K2" s="28" t="s">
-        <v>134</v>
-      </c>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="20"/>
+      <c r="A2" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="16"/>
+      <c r="F2" s="26" t="s">
+        <v>129</v>
+      </c>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="16"/>
+      <c r="K2" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15"/>
+      <c r="N2" s="16"/>
     </row>
     <row r="3" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="21"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="22"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="22"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="22"/>
+      <c r="A3" s="17"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="18"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="18"/>
+      <c r="K3" s="17"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="18"/>
     </row>
     <row r="4" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="23"/>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="25"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="25"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="24"/>
-      <c r="M4" s="24"/>
-      <c r="N4" s="25"/>
+      <c r="A4" s="19"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="21"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="21"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="20"/>
+      <c r="N4" s="21"/>
     </row>
     <row r="5" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="6" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="31" t="s">
-        <v>135</v>
-      </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="20"/>
-      <c r="F6" s="18" t="s">
-        <v>136</v>
-      </c>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="20"/>
-      <c r="K6" s="26" t="s">
-        <v>137</v>
-      </c>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="20"/>
+      <c r="A6" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="16"/>
+      <c r="F6" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="16"/>
+      <c r="K6" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="16"/>
     </row>
     <row r="7" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="21"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="22"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="22"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="22"/>
+      <c r="A7" s="17"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="18"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="18"/>
+      <c r="K7" s="17"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="18"/>
     </row>
     <row r="8" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="23"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="25"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="25"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="24"/>
-      <c r="M8" s="24"/>
-      <c r="N8" s="25"/>
+      <c r="A8" s="19"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="21"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="21"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="20"/>
+      <c r="N8" s="21"/>
     </row>
     <row r="9" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="10" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="11" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="29" t="s">
-        <v>138</v>
-      </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="20"/>
+      <c r="A11" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="16"/>
     </row>
     <row r="12" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="21"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="22"/>
+      <c r="A12" s="17"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="18"/>
     </row>
     <row r="13" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="21"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="22"/>
+      <c r="A13" s="17"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="18"/>
     </row>
     <row r="14" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="23"/>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="25"/>
+      <c r="A14" s="19"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="21"/>
     </row>
     <row r="15" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.35"/>

</xml_diff>